<commit_message>
arbon Credits adjustments: editable inputs, baseline checks for calculations. And other fixes like change in units of tariff and upstream values
</commit_message>
<xml_diff>
--- a/backend/Rwanda/capex-fuels-Aligned.xlsx
+++ b/backend/Rwanda/capex-fuels-Aligned.xlsx
@@ -973,16 +973,16 @@
         <v>32.10847138103129</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>28.93579531449316</v>
+        <v>32.39487560125811</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>22.8474653855744</v>
+        <v>32.42652479692517</v>
       </c>
       <c r="M10" s="7" t="n">
-        <v>16.98862229061014</v>
+        <v>32.20454263639458</v>
       </c>
       <c r="N10" s="7" t="n">
-        <v>11.28461652587229</v>
+        <v>28.19750607481915</v>
       </c>
     </row>
   </sheetData>
@@ -1502,34 +1502,34 @@
         <v>514.6788571428572</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>781.8227641112045</v>
+        <v>782.7908571428571</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>1038.788227869545</v>
+        <v>1039.729428571429</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>1284.695422509105</v>
+        <v>1285.607142857143</v>
       </c>
       <c r="I10" s="14" t="n">
-        <v>1519.655476435358</v>
+        <v>1519.567621254061</v>
       </c>
       <c r="J10" s="14" t="n">
-        <v>1802.423532484009</v>
+        <v>1802.329942155259</v>
       </c>
       <c r="K10" s="14" t="n">
-        <v>2130.499616348119</v>
+        <v>2130.402851080533</v>
       </c>
       <c r="L10" s="14" t="n">
-        <v>2209.051191978977</v>
+        <v>2443.269190721073</v>
       </c>
       <c r="M10" s="14" t="n">
-        <v>2227.420997187764</v>
+        <v>2741.070675341151</v>
       </c>
       <c r="N10" s="14" t="n">
-        <v>2242.167162521164</v>
+        <v>3023.967330633833</v>
       </c>
       <c r="O10" s="14" t="n">
-        <v>2134.384961520787</v>
+        <v>2938.841763407548</v>
       </c>
     </row>
     <row r="11">
@@ -2032,34 +2032,34 @@
         <v>83.7564</v>
       </c>
       <c r="F20" s="14" t="n">
-        <v>127.3999169978782</v>
+        <v>127.4044</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>168.6090150617134</v>
+        <v>168.6152</v>
       </c>
       <c r="H20" s="14" t="n">
-        <v>207.4037787098245</v>
+        <v>207.4084</v>
       </c>
       <c r="I20" s="14" t="n">
-        <v>243.8084432863687</v>
+        <v>243.8087169978782</v>
       </c>
       <c r="J20" s="14" t="n">
-        <v>249.1909977820617</v>
+        <v>249.1866150617134</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>225.181987297712</v>
+        <v>225.1781787098245</v>
       </c>
       <c r="L20" s="14" t="n">
-        <v>164.1567406475907</v>
+        <v>201.7932432863687</v>
       </c>
       <c r="M20" s="14" t="n">
-        <v>95.2742584119942</v>
+        <v>179.0217977820617</v>
       </c>
       <c r="N20" s="14" t="n">
-        <v>29.46555867771927</v>
+        <v>156.863587297712</v>
       </c>
       <c r="O20" s="14" t="n">
-        <v>-20.88739638024723</v>
+        <v>110.0771406475907</v>
       </c>
     </row>
   </sheetData>
@@ -2149,40 +2149,40 @@
         </is>
       </c>
       <c r="D2" s="14" t="n">
-        <v>214.8070553210895</v>
+        <v>214.81</v>
       </c>
       <c r="E2" s="14" t="n">
-        <v>248.020871355366</v>
+        <v>248.02</v>
       </c>
       <c r="F2" s="14" t="n">
-        <v>245.5406626418123</v>
+        <v>245.54</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>243.0852560153942</v>
+        <v>243.09</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>240.6544034552403</v>
+        <v>240.65</v>
       </c>
       <c r="I2" s="14" t="n">
-        <v>238.2478594206879</v>
+        <v>238.25</v>
       </c>
       <c r="J2" s="14" t="n">
-        <v>273.9304205498366</v>
+        <v>273.93</v>
       </c>
       <c r="K2" s="14" t="n">
-        <v>309.0653526620416</v>
+        <v>309.07</v>
       </c>
       <c r="L2" s="14" t="n">
-        <v>305.9746991354211</v>
+        <v>305.97</v>
       </c>
       <c r="M2" s="14" t="n">
-        <v>302.914952144067</v>
+        <v>302.91</v>
       </c>
       <c r="N2" s="14" t="n">
-        <v>299.8858026226263</v>
+        <v>299.89</v>
       </c>
       <c r="O2" s="14" t="n">
-        <v>206.371686125674</v>
+        <v>206.37</v>
       </c>
     </row>
     <row r="3" ht="15.5" customHeight="1">
@@ -2202,40 +2202,40 @@
         </is>
       </c>
       <c r="D3" s="14" t="n">
-        <v>214.8070553210895</v>
+        <v>214.81</v>
       </c>
       <c r="E3" s="14" t="n">
-        <v>462.8279266764555</v>
+        <v>462.83</v>
       </c>
       <c r="F3" s="14" t="n">
-        <v>708.3685893182678</v>
+        <v>708.37</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>951.453845333662</v>
+        <v>951.46</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>1192.108248788902</v>
+        <v>1192.11</v>
       </c>
       <c r="I3" s="14" t="n">
-        <v>1430.35610820959</v>
+        <v>1430.36</v>
       </c>
       <c r="J3" s="14" t="n">
-        <v>1704.286528759427</v>
+        <v>1704.29</v>
       </c>
       <c r="K3" s="14" t="n">
-        <v>2013.351881421469</v>
+        <v>2013.36</v>
       </c>
       <c r="L3" s="14" t="n">
-        <v>2319.326580556889</v>
+        <v>2319.33</v>
       </c>
       <c r="M3" s="14" t="n">
-        <v>2622.241532700957</v>
+        <v>2622.24</v>
       </c>
       <c r="N3" s="14" t="n">
-        <v>2922.127335323583</v>
+        <v>2922.13</v>
       </c>
       <c r="O3" s="14" t="n">
-        <v>3128.499021449257</v>
+        <v>3128.5</v>
       </c>
     </row>
     <row r="4" ht="15.5" customHeight="1">
@@ -2255,7 +2255,7 @@
         </is>
       </c>
       <c r="D4" s="14" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>0</v>
@@ -2308,40 +2308,40 @@
         </is>
       </c>
       <c r="D5" s="14" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="E5" s="14" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="F5" s="14" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I5" s="14" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="J5" s="14" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="K5" s="14" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="L5" s="14" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="M5" s="14" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="N5" s="14" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="O5" s="14" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" ht="15.5" customHeight="1">
@@ -2361,40 +2361,40 @@
         </is>
       </c>
       <c r="D6" s="14" t="n">
-        <v>213.8070553210895</v>
+        <v>214.81</v>
       </c>
       <c r="E6" s="14" t="n">
-        <v>248.020871355366</v>
+        <v>248.02</v>
       </c>
       <c r="F6" s="14" t="n">
-        <v>245.5406626418123</v>
+        <v>245.54</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>243.0852560153942</v>
+        <v>243.09</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>240.6544034552403</v>
+        <v>240.65</v>
       </c>
       <c r="I6" s="14" t="n">
-        <v>238.2478594206879</v>
+        <v>238.25</v>
       </c>
       <c r="J6" s="14" t="n">
-        <v>273.9304205498366</v>
+        <v>273.93</v>
       </c>
       <c r="K6" s="14" t="n">
-        <v>309.0653526620416</v>
+        <v>309.07</v>
       </c>
       <c r="L6" s="14" t="n">
-        <v>305.9746991354211</v>
+        <v>305.97</v>
       </c>
       <c r="M6" s="14" t="n">
-        <v>302.914952144067</v>
+        <v>302.91</v>
       </c>
       <c r="N6" s="14" t="n">
-        <v>299.8858026226263</v>
+        <v>299.89</v>
       </c>
       <c r="O6" s="14" t="n">
-        <v>206.371686125674</v>
+        <v>206.37</v>
       </c>
     </row>
     <row r="7" ht="15.5" customHeight="1">
@@ -2414,40 +2414,40 @@
         </is>
       </c>
       <c r="D7" s="14" t="n">
-        <v>213.8070553210895</v>
+        <v>214.81</v>
       </c>
       <c r="E7" s="14" t="n">
-        <v>461.8279266764555</v>
+        <v>462.83</v>
       </c>
       <c r="F7" s="14" t="n">
-        <v>707.3685893182678</v>
+        <v>708.37</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>950.453845333662</v>
+        <v>951.46</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>1191.108248788902</v>
+        <v>1192.11</v>
       </c>
       <c r="I7" s="14" t="n">
-        <v>1429.35610820959</v>
+        <v>1430.36</v>
       </c>
       <c r="J7" s="14" t="n">
-        <v>1703.286528759427</v>
+        <v>1704.29</v>
       </c>
       <c r="K7" s="14" t="n">
-        <v>2012.351881421469</v>
+        <v>2013.36</v>
       </c>
       <c r="L7" s="14" t="n">
-        <v>2318.326580556889</v>
+        <v>2319.33</v>
       </c>
       <c r="M7" s="14" t="n">
-        <v>2621.241532700957</v>
+        <v>2622.24</v>
       </c>
       <c r="N7" s="14" t="n">
-        <v>2921.127335323583</v>
+        <v>2922.13</v>
       </c>
       <c r="O7" s="14" t="n">
-        <v>3127.499021449257</v>
+        <v>3128.5</v>
       </c>
     </row>
     <row r="8" ht="15.5" customHeight="1">
@@ -2520,40 +2520,40 @@
         </is>
       </c>
       <c r="D9" s="14" t="n">
-        <v>6.108773009173986</v>
+        <v>6.137428571428572</v>
       </c>
       <c r="E9" s="14" t="n">
-        <v>13.1950836193273</v>
+        <v>13.22371428571429</v>
       </c>
       <c r="F9" s="14" t="n">
-        <v>20.21053112337908</v>
+        <v>20.23914285714286</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>27.15582415239034</v>
+        <v>27.18457142857143</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>34.03166425111149</v>
+        <v>34.06028571428572</v>
       </c>
       <c r="I9" s="14" t="n">
-        <v>40.83874594884544</v>
+        <v>40.86742857142858</v>
       </c>
       <c r="J9" s="14" t="n">
-        <v>48.66532939312648</v>
+        <v>48.694</v>
       </c>
       <c r="K9" s="14" t="n">
-        <v>57.49576804061338</v>
+        <v>57.52457142857143</v>
       </c>
       <c r="L9" s="14" t="n">
-        <v>66.23790230162541</v>
+        <v>66.26657142857142</v>
       </c>
       <c r="M9" s="14" t="n">
-        <v>74.89261522002734</v>
+        <v>74.92114285714285</v>
       </c>
       <c r="N9" s="14" t="n">
-        <v>83.46078100924522</v>
+        <v>83.48942857142856</v>
       </c>
       <c r="O9" s="14" t="n">
-        <v>89.35711489855019</v>
+        <v>89.38571428571427</v>
       </c>
     </row>
     <row r="10" ht="15.5" customHeight="1">
@@ -2573,40 +2573,40 @@
         </is>
       </c>
       <c r="D10" s="14" t="n">
-        <v>207.6982823119155</v>
+        <v>208.6725714285714</v>
       </c>
       <c r="E10" s="14" t="n">
-        <v>442.5240700479542</v>
+        <v>443.4688571428571</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>667.8542015663875</v>
+        <v>668.7697142857143</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>883.7836334293913</v>
+        <v>883.7008537404871</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>1090.40637263352</v>
+        <v>1090.320070047954</v>
       </c>
       <c r="I10" s="14" t="n">
-        <v>1287.815486105363</v>
+        <v>1287.731915852102</v>
       </c>
       <c r="J10" s="14" t="n">
-        <v>1513.080577262073</v>
+        <v>1512.991919143678</v>
       </c>
       <c r="K10" s="14" t="n">
-        <v>1764.650161883501</v>
+        <v>1764.57037263352</v>
       </c>
       <c r="L10" s="14" t="n">
-        <v>1796.688676405381</v>
+        <v>2004.300343248221</v>
       </c>
       <c r="M10" s="14" t="n">
-        <v>1789.885225593382</v>
+        <v>2232.318291547787</v>
       </c>
       <c r="N10" s="14" t="n">
-        <v>1780.98011568833</v>
+        <v>2448.743019026359</v>
       </c>
       <c r="O10" s="14" t="n">
-        <v>1682.065255052449</v>
+        <v>2358.062390691095</v>
       </c>
     </row>
     <row r="11">
@@ -2679,40 +2679,40 @@
         </is>
       </c>
       <c r="D12" s="14" t="n">
-        <v>39.20533020612309</v>
+        <v>39.21</v>
       </c>
       <c r="E12" s="14" t="n">
-        <v>49.66803257508351</v>
+        <v>49.67</v>
       </c>
       <c r="F12" s="14" t="n">
-        <v>49.17135224933267</v>
+        <v>49.17</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>48.67963872683934</v>
+        <v>48.68</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>48.19284233957096</v>
+        <v>48.19</v>
       </c>
       <c r="I12" s="14" t="n">
-        <v>47.71091391617525</v>
+        <v>47.71</v>
       </c>
       <c r="J12" s="14" t="n">
-        <v>17.3764528627935</v>
+        <v>17.38</v>
       </c>
       <c r="K12" s="14" t="n">
-        <v>-12.50500172575464</v>
+        <v>-12.51</v>
       </c>
       <c r="L12" s="14" t="n">
-        <v>-12.37995170849709</v>
+        <v>-12.38</v>
       </c>
       <c r="M12" s="14" t="n">
-        <v>-12.25615219141212</v>
+        <v>-12.26</v>
       </c>
       <c r="N12" s="14" t="n">
-        <v>-12.133590669498</v>
+        <v>-12.13</v>
       </c>
       <c r="O12" s="14" t="n">
-        <v>0.9231042276977806</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="13" ht="15.5" customHeight="1">
@@ -2732,40 +2732,40 @@
         </is>
       </c>
       <c r="D13" s="14" t="n">
-        <v>39.20533020612309</v>
+        <v>39.21</v>
       </c>
       <c r="E13" s="14" t="n">
-        <v>88.87336278120659</v>
+        <v>88.88</v>
       </c>
       <c r="F13" s="14" t="n">
-        <v>138.0447150305393</v>
+        <v>138.05</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>186.7243537573786</v>
+        <v>186.73</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>234.9171960969496</v>
+        <v>234.92</v>
       </c>
       <c r="I13" s="14" t="n">
-        <v>282.6281100131248</v>
+        <v>282.63</v>
       </c>
       <c r="J13" s="14" t="n">
-        <v>300.0045628759183</v>
+        <v>300.01</v>
       </c>
       <c r="K13" s="14" t="n">
-        <v>287.4995611501636</v>
+        <v>287.5</v>
       </c>
       <c r="L13" s="14" t="n">
-        <v>275.1196094416665</v>
+        <v>275.12</v>
       </c>
       <c r="M13" s="14" t="n">
-        <v>262.8634572502544</v>
+        <v>262.86</v>
       </c>
       <c r="N13" s="14" t="n">
-        <v>250.7298665807564</v>
+        <v>250.73</v>
       </c>
       <c r="O13" s="14" t="n">
-        <v>251.6529708084542</v>
+        <v>251.65</v>
       </c>
     </row>
     <row r="14" ht="15.5" customHeight="1">
@@ -2891,40 +2891,40 @@
         </is>
       </c>
       <c r="D16" s="14" t="n">
-        <v>39.20533020612309</v>
+        <v>39.21</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>49.66803257508351</v>
+        <v>49.67</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>49.17135224933267</v>
+        <v>49.17</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>48.67963872683934</v>
+        <v>48.68</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>48.19284233957096</v>
+        <v>48.19</v>
       </c>
       <c r="I16" s="14" t="n">
-        <v>47.71091391617525</v>
+        <v>47.71</v>
       </c>
       <c r="J16" s="14" t="n">
-        <v>17.3764528627935</v>
+        <v>17.38</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>-12.50500172575464</v>
+        <v>-12.51</v>
       </c>
       <c r="L16" s="14" t="n">
-        <v>-12.37995170849709</v>
+        <v>-12.38</v>
       </c>
       <c r="M16" s="14" t="n">
-        <v>-12.25615219141212</v>
+        <v>-12.26</v>
       </c>
       <c r="N16" s="14" t="n">
-        <v>-12.133590669498</v>
+        <v>-12.13</v>
       </c>
       <c r="O16" s="14" t="n">
-        <v>0.9231042276977806</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="17" ht="15.5" customHeight="1">
@@ -2944,40 +2944,40 @@
         </is>
       </c>
       <c r="D17" s="14" t="n">
-        <v>39.20533020612309</v>
+        <v>39.21</v>
       </c>
       <c r="E17" s="14" t="n">
-        <v>88.87336278120659</v>
+        <v>88.88</v>
       </c>
       <c r="F17" s="14" t="n">
-        <v>138.0447150305393</v>
+        <v>138.05</v>
       </c>
       <c r="G17" s="14" t="n">
-        <v>186.7243537573786</v>
+        <v>186.73</v>
       </c>
       <c r="H17" s="14" t="n">
-        <v>234.9171960969496</v>
+        <v>234.92</v>
       </c>
       <c r="I17" s="14" t="n">
-        <v>282.6281100131248</v>
+        <v>282.63</v>
       </c>
       <c r="J17" s="14" t="n">
-        <v>300.0045628759183</v>
+        <v>300.01</v>
       </c>
       <c r="K17" s="14" t="n">
-        <v>287.4995611501636</v>
+        <v>287.5</v>
       </c>
       <c r="L17" s="14" t="n">
-        <v>275.1196094416665</v>
+        <v>275.12</v>
       </c>
       <c r="M17" s="14" t="n">
-        <v>262.8634572502544</v>
+        <v>262.86</v>
       </c>
       <c r="N17" s="14" t="n">
-        <v>250.7298665807564</v>
+        <v>250.73</v>
       </c>
       <c r="O17" s="14" t="n">
-        <v>251.6529708084542</v>
+        <v>251.65</v>
       </c>
     </row>
     <row r="18" ht="15.5" customHeight="1">
@@ -3050,40 +3050,40 @@
         </is>
       </c>
       <c r="D19" s="14" t="n">
-        <v>1.568213208244923</v>
+        <v>1.5684</v>
       </c>
       <c r="E19" s="14" t="n">
-        <v>3.554934511248264</v>
+        <v>3.5552</v>
       </c>
       <c r="F19" s="14" t="n">
-        <v>5.52178860122157</v>
+        <v>5.522</v>
       </c>
       <c r="G19" s="14" t="n">
-        <v>7.468974150295144</v>
+        <v>7.469200000000001</v>
       </c>
       <c r="H19" s="14" t="n">
-        <v>9.396687843877983</v>
+        <v>9.396800000000001</v>
       </c>
       <c r="I19" s="14" t="n">
-        <v>11.30512440052499</v>
+        <v>11.3052</v>
       </c>
       <c r="J19" s="14" t="n">
-        <v>12.00018251503673</v>
+        <v>12.0004</v>
       </c>
       <c r="K19" s="14" t="n">
-        <v>11.49998244600654</v>
+        <v>11.5</v>
       </c>
       <c r="L19" s="14" t="n">
-        <v>11.00478437766666</v>
+        <v>11.0048</v>
       </c>
       <c r="M19" s="14" t="n">
-        <v>10.51453829001018</v>
+        <v>10.5144</v>
       </c>
       <c r="N19" s="14" t="n">
-        <v>10.02919466323026</v>
+        <v>10.0292</v>
       </c>
       <c r="O19" s="14" t="n">
-        <v>10.06611883233817</v>
+        <v>10.066</v>
       </c>
     </row>
     <row r="20" ht="15.5" customHeight="1">
@@ -3103,40 +3103,40 @@
         </is>
       </c>
       <c r="D20" s="14" t="n">
-        <v>37.63711699787817</v>
+        <v>37.6416</v>
       </c>
       <c r="E20" s="14" t="n">
-        <v>83.75021506171342</v>
+        <v>83.7564</v>
       </c>
       <c r="F20" s="14" t="n">
-        <v>127.3997787098245</v>
+        <v>127.4044</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>168.6104432863687</v>
+        <v>168.6107169978782</v>
       </c>
       <c r="H20" s="14" t="n">
-        <v>207.4065977820617</v>
+        <v>207.4022150617134</v>
       </c>
       <c r="I20" s="14" t="n">
-        <v>243.812387297712</v>
+        <v>243.8085787098245</v>
       </c>
       <c r="J20" s="14" t="n">
-        <v>249.1886576454688</v>
+        <v>249.1880432863687</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>225.1836734737076</v>
+        <v>225.1809977820617</v>
       </c>
       <c r="L20" s="14" t="n">
-        <v>164.1618203896658</v>
+        <v>201.797187297712</v>
       </c>
       <c r="M20" s="14" t="n">
-        <v>95.2780318444082</v>
+        <v>179.0194576454688</v>
       </c>
       <c r="N20" s="14" t="n">
-        <v>29.46568286356872</v>
+        <v>156.8652734737076</v>
       </c>
       <c r="O20" s="14" t="n">
-        <v>-20.88799631761588</v>
+        <v>110.0822203896658</v>
       </c>
     </row>
   </sheetData>

</xml_diff>